<commit_message>
el logo fuciona, las bajas e importaciones igual
</commit_message>
<xml_diff>
--- a/src/assets/Usuarios de crownparadise.xlsx
+++ b/src/assets/Usuarios de crownparadise.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66420935-A5D1-4241-93E0-48C7B6953AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E460E8-0B8E-4F1D-8A4B-009CEED57766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="285">
   <si>
     <t>Nombre</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Capital Humano</t>
   </si>
   <si>
-    <t>CROWNCUN\asistenterh</t>
-  </si>
-  <si>
     <t>Asistente de Almacén</t>
   </si>
   <si>
@@ -326,9 +323,6 @@
     <t/>
   </si>
   <si>
-    <t>LOCAL\nitro</t>
-  </si>
-  <si>
     <t>Eduardo Espinola</t>
   </si>
   <si>
@@ -509,15 +503,9 @@
     <t>Lock Service 1</t>
   </si>
   <si>
-    <t>LOCAL\lockservice</t>
-  </si>
-  <si>
     <t>Lock Service 2</t>
   </si>
   <si>
-    <t>LOCAL\locklink</t>
-  </si>
-  <si>
     <t>CROWNCUN\jefecompras</t>
   </si>
   <si>
@@ -566,9 +554,6 @@
     <t>mantenimientocun@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\asistmanto</t>
-  </si>
-  <si>
     <t>Mensajero Contabilidad</t>
   </si>
   <si>
@@ -716,9 +701,6 @@
     <t>mantenimientocun3@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\mantenimiento</t>
-  </si>
-  <si>
     <t>Teatro Yumik</t>
   </si>
   <si>
@@ -743,9 +725,6 @@
     <t>mantenimientocun2@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\mantenimientocun</t>
-  </si>
-  <si>
     <t>Urayma Isea</t>
   </si>
   <si>
@@ -773,9 +752,6 @@
     <t>practicascostos@crownparadise.com</t>
   </si>
   <si>
-    <t>LOCAL\practicas</t>
-  </si>
-  <si>
     <t>Es jefe</t>
   </si>
   <si>
@@ -827,12 +803,6 @@
     <t>ARRIVA\gscun09</t>
   </si>
   <si>
-    <t>LOCAL\sala de ventas</t>
-  </si>
-  <si>
-    <t>LOCAL\atencion a socios</t>
-  </si>
-  <si>
     <t>ARRIVA\gscun11</t>
   </si>
   <si>
@@ -885,6 +855,21 @@
   </si>
   <si>
     <t>ARRIVA\apublicascun</t>
+  </si>
+  <si>
+    <t>ARRIVA\asiscpcun</t>
+  </si>
+  <si>
+    <t>ARRIVA\asisacpcun</t>
+  </si>
+  <si>
+    <t>ARRIVA\asismantocun</t>
+  </si>
+  <si>
+    <t>ARRIVA\mantenimientocun</t>
+  </si>
+  <si>
+    <t>ARRIVA\mantenimientocun02</t>
   </si>
 </sst>
 </file>
@@ -950,16 +935,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -999,8 +985,8 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}" name="Tabla1" displayName="Tabla1" ref="A1:F92" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:F92" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E81">
-    <sortCondition ref="D1:D81"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F92">
+    <sortCondition ref="D1:D92"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9490AABE-096E-46D2-A730-536117DCF14A}" name="Nombre"/>
@@ -1364,207 +1350,204 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" t="s">
         <v>115</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E2" t="s">
         <v>116</v>
       </c>
-      <c r="C2" t="s">
-        <v>117</v>
-      </c>
-      <c r="D2" t="s">
-        <v>117</v>
-      </c>
-      <c r="E2" t="s">
-        <v>118</v>
-      </c>
       <c r="F2" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>120</v>
+      </c>
+      <c r="B3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E3" t="s">
         <v>122</v>
       </c>
-      <c r="B3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C3" t="s">
-        <v>117</v>
-      </c>
-      <c r="D3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E3" t="s">
-        <v>124</v>
-      </c>
       <c r="F3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" t="s">
+        <v>115</v>
+      </c>
+      <c r="E4" t="s">
         <v>129</v>
       </c>
-      <c r="B4" t="s">
-        <v>130</v>
-      </c>
-      <c r="C4" t="s">
-        <v>117</v>
-      </c>
-      <c r="D4" t="s">
-        <v>117</v>
-      </c>
-      <c r="E4" t="s">
-        <v>131</v>
-      </c>
       <c r="F4" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E5" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="F5" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B6" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="F6" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="B7" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="C7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E7" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="F7" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>36</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" t="s">
         <v>37</v>
       </c>
-      <c r="D8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" t="s">
-        <v>38</v>
-      </c>
       <c r="F8" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B9" t="s">
         <v>101</v>
       </c>
-      <c r="B9" t="s">
-        <v>102</v>
-      </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E9" t="s">
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B10" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F10" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B11" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="F11" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1581,18 +1564,18 @@
         <v>29</v>
       </c>
       <c r="E12" t="s">
-        <v>30</v>
+        <v>280</v>
       </c>
       <c r="F12" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" t="s">
         <v>39</v>
-      </c>
-      <c r="B13" t="s">
-        <v>40</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
@@ -1601,18 +1584,18 @@
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>281</v>
       </c>
       <c r="F13" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
         <v>76</v>
-      </c>
-      <c r="B14" t="s">
-        <v>77</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -1621,18 +1604,18 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F14" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B15" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
@@ -1641,18 +1624,18 @@
         <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F15" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C16" t="s">
         <v>29</v>
@@ -1661,18 +1644,18 @@
         <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F16" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B17" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C17" t="s">
         <v>29</v>
@@ -1681,10 +1664,10 @@
         <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F17" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -1704,7 +1687,7 @@
         <v>17</v>
       </c>
       <c r="F18" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -1724,35 +1707,35 @@
         <v>20</v>
       </c>
       <c r="F19" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
         <v>31</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>32</v>
-      </c>
-      <c r="C20" t="s">
-        <v>33</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>45</v>
+      </c>
+      <c r="B21" t="s">
         <v>46</v>
-      </c>
-      <c r="B21" t="s">
-        <v>47</v>
       </c>
       <c r="C21" t="s">
         <v>15</v>
@@ -1761,18 +1744,18 @@
         <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F21" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>48</v>
+      </c>
+      <c r="B22" t="s">
         <v>49</v>
-      </c>
-      <c r="B22" t="s">
-        <v>50</v>
       </c>
       <c r="C22" t="s">
         <v>15</v>
@@ -1781,18 +1764,18 @@
         <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F22" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" t="s">
         <v>70</v>
-      </c>
-      <c r="B23" t="s">
-        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>15</v>
@@ -1801,58 +1784,58 @@
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F23" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" t="s">
         <v>79</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>80</v>
-      </c>
-      <c r="C24" t="s">
-        <v>81</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F24" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" t="s">
         <v>87</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>88</v>
-      </c>
-      <c r="C25" t="s">
-        <v>89</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F25" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C26" t="s">
         <v>15</v>
@@ -1861,18 +1844,18 @@
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F26" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B27" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C27" t="s">
         <v>15</v>
@@ -1881,98 +1864,98 @@
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F27" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>123</v>
+      </c>
+      <c r="B28" t="s">
+        <v>124</v>
+      </c>
+      <c r="C28" t="s">
         <v>125</v>
-      </c>
-      <c r="B28" t="s">
-        <v>126</v>
-      </c>
-      <c r="C28" t="s">
-        <v>127</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F28" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B29" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F29" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>144</v>
+      </c>
+      <c r="B30" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" t="s">
         <v>146</v>
-      </c>
-      <c r="B30" t="s">
-        <v>147</v>
-      </c>
-      <c r="C30" t="s">
-        <v>148</v>
       </c>
       <c r="D30" t="s">
         <v>16</v>
       </c>
       <c r="E30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F30" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="C31" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D31" t="s">
         <v>16</v>
       </c>
       <c r="E31" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F31" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B32" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C32" t="s">
         <v>15</v>
@@ -1981,18 +1964,18 @@
         <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="F32" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B33" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C33" t="s">
         <v>15</v>
@@ -2001,38 +1984,38 @@
         <v>16</v>
       </c>
       <c r="E33" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="F33" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B34" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D34" t="s">
         <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F34" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
         <v>15</v>
@@ -2041,38 +2024,38 @@
         <v>16</v>
       </c>
       <c r="E35" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="F35" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="B36" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C36" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D36" t="s">
         <v>16</v>
       </c>
       <c r="E36" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="F36" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B37" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C37" t="s">
         <v>15</v>
@@ -2081,58 +2064,55 @@
         <v>16</v>
       </c>
       <c r="E37" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="F37" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="B38" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="C38" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="D38" t="s">
         <v>16</v>
       </c>
       <c r="E38" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="F38" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>21</v>
-      </c>
-      <c r="B39" t="s">
-        <v>22</v>
+        <v>243</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>244</v>
       </c>
       <c r="C39" t="s">
-        <v>23</v>
+        <v>238</v>
       </c>
       <c r="D39" t="s">
-        <v>24</v>
-      </c>
-      <c r="E39" t="s">
-        <v>287</v>
+        <v>16</v>
       </c>
       <c r="F39" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B40" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C40" t="s">
         <v>23</v>
@@ -2141,1063 +2121,1051 @@
         <v>24</v>
       </c>
       <c r="E40" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="F40" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="C41" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="D41" t="s">
         <v>24</v>
       </c>
       <c r="E41" t="s">
-        <v>55</v>
+        <v>276</v>
       </c>
       <c r="F41" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B42" t="s">
+        <v>52</v>
+      </c>
+      <c r="C42" t="s">
         <v>53</v>
-      </c>
-      <c r="C42" t="s">
-        <v>54</v>
       </c>
       <c r="D42" t="s">
         <v>24</v>
       </c>
       <c r="E42" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="F42" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B43" t="s">
+        <v>52</v>
+      </c>
+      <c r="C43" t="s">
         <v>53</v>
-      </c>
-      <c r="C43" t="s">
-        <v>54</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
       </c>
       <c r="E43" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F43" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B44" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" t="s">
         <v>53</v>
-      </c>
-      <c r="C44" t="s">
-        <v>54</v>
       </c>
       <c r="D44" t="s">
         <v>24</v>
       </c>
       <c r="E44" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="F44" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B45" t="s">
+        <v>52</v>
+      </c>
+      <c r="C45" t="s">
         <v>53</v>
-      </c>
-      <c r="C45" t="s">
-        <v>54</v>
       </c>
       <c r="D45" t="s">
         <v>24</v>
       </c>
       <c r="E45" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="F45" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B46" t="s">
+        <v>52</v>
+      </c>
+      <c r="C46" t="s">
         <v>53</v>
-      </c>
-      <c r="C46" t="s">
-        <v>54</v>
       </c>
       <c r="D46" t="s">
         <v>24</v>
       </c>
       <c r="E46" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F46" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B47" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="C47" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="D47" t="s">
         <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F47" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B48" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="C48" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D48" t="s">
         <v>24</v>
       </c>
       <c r="E48" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="F48" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="B49" t="s">
+        <v>73</v>
+      </c>
+      <c r="C49" t="s">
         <v>67</v>
-      </c>
-      <c r="C49" t="s">
-        <v>68</v>
       </c>
       <c r="D49" t="s">
         <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="F49" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B50" t="s">
+        <v>66</v>
+      </c>
+      <c r="C50" t="s">
         <v>67</v>
-      </c>
-      <c r="C50" t="s">
-        <v>68</v>
       </c>
       <c r="D50" t="s">
         <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F50" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B51" t="s">
-        <v>99</v>
+        <v>66</v>
       </c>
       <c r="C51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D51" t="s">
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F51" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>110</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>249</v>
+        <v>97</v>
+      </c>
+      <c r="B52" t="s">
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="D52" t="s">
         <v>24</v>
       </c>
       <c r="E52" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="F52" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>119</v>
-      </c>
-      <c r="B53" t="s">
-        <v>120</v>
+        <v>108</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>242</v>
       </c>
       <c r="C53" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="D53" t="s">
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>121</v>
+        <v>109</v>
       </c>
       <c r="F53" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>132</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>74</v>
+        <v>117</v>
+      </c>
+      <c r="B54" t="s">
+        <v>118</v>
       </c>
       <c r="C54" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="D54" t="s">
         <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="F54" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>136</v>
-      </c>
-      <c r="B55" t="s">
-        <v>137</v>
+        <v>130</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>73</v>
       </c>
       <c r="C55" t="s">
-        <v>138</v>
+        <v>53</v>
       </c>
       <c r="D55" t="s">
         <v>24</v>
       </c>
       <c r="E55" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="F55" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="B56" t="s">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="C56" t="s">
-        <v>151</v>
+        <v>136</v>
       </c>
       <c r="D56" t="s">
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="F56" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="B57" t="s">
-        <v>161</v>
+        <v>101</v>
       </c>
       <c r="C57" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D57" t="s">
         <v>24</v>
       </c>
       <c r="E57" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="F57" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B58" t="s">
-        <v>102</v>
+        <v>159</v>
       </c>
       <c r="C58" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D58" t="s">
         <v>24</v>
       </c>
       <c r="E58" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="F58" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C59" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D59" t="s">
         <v>24</v>
       </c>
-      <c r="E59" t="s">
-        <v>166</v>
-      </c>
       <c r="F59" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s">
-        <v>175</v>
+        <v>101</v>
       </c>
       <c r="C60" t="s">
-        <v>176</v>
+        <v>149</v>
       </c>
       <c r="D60" t="s">
         <v>24</v>
       </c>
-      <c r="E60" t="s">
-        <v>177</v>
-      </c>
       <c r="F60" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="B61" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="C61" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="D61" t="s">
         <v>24</v>
       </c>
-      <c r="E61" s="4" t="s">
-        <v>289</v>
+      <c r="E61" t="s">
+        <v>173</v>
       </c>
       <c r="F61" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>228</v>
+        <v>185</v>
       </c>
       <c r="B62" t="s">
-        <v>229</v>
+        <v>186</v>
       </c>
       <c r="C62" t="s">
-        <v>54</v>
+        <v>187</v>
       </c>
       <c r="D62" t="s">
         <v>24</v>
       </c>
-      <c r="E62" t="s">
-        <v>230</v>
+      <c r="E62" s="3" t="s">
+        <v>279</v>
       </c>
       <c r="F62" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>237</v>
+        <v>223</v>
       </c>
       <c r="B63" t="s">
-        <v>238</v>
+        <v>224</v>
       </c>
       <c r="C63" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
       <c r="D63" t="s">
         <v>24</v>
       </c>
       <c r="E63" t="s">
-        <v>239</v>
+        <v>225</v>
       </c>
       <c r="F63" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>186</v>
+        <v>231</v>
       </c>
       <c r="B64" t="s">
-        <v>187</v>
+        <v>232</v>
       </c>
       <c r="C64" t="s">
-        <v>188</v>
+        <v>23</v>
       </c>
       <c r="D64" t="s">
-        <v>188</v>
+        <v>24</v>
       </c>
       <c r="E64" t="s">
-        <v>189</v>
+        <v>233</v>
       </c>
       <c r="F64" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>200</v>
+        <v>181</v>
       </c>
       <c r="B65" t="s">
-        <v>201</v>
+        <v>182</v>
       </c>
       <c r="C65" t="s">
-        <v>202</v>
+        <v>183</v>
       </c>
       <c r="D65" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="E65" t="s">
-        <v>203</v>
+        <v>184</v>
       </c>
       <c r="F65" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>42</v>
+        <v>195</v>
       </c>
       <c r="B66" t="s">
-        <v>43</v>
+        <v>196</v>
       </c>
       <c r="C66" t="s">
-        <v>44</v>
+        <v>197</v>
       </c>
       <c r="D66" t="s">
-        <v>44</v>
+        <v>183</v>
       </c>
       <c r="E66" t="s">
-        <v>45</v>
+        <v>198</v>
       </c>
       <c r="F66" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>112</v>
-      </c>
-      <c r="B67" t="s">
-        <v>113</v>
+        <v>249</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>271</v>
       </c>
       <c r="C67" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="D67" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="E67" t="s">
-        <v>114</v>
+        <v>257</v>
       </c>
       <c r="F67" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>181</v>
-      </c>
-      <c r="B68" t="s">
-        <v>182</v>
+        <v>250</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>265</v>
       </c>
       <c r="C68" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="D68" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="E68" t="s">
-        <v>183</v>
+        <v>258</v>
       </c>
       <c r="F68" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>231</v>
-      </c>
-      <c r="B69" t="s">
-        <v>232</v>
+        <v>251</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>272</v>
       </c>
       <c r="C69" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="D69" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="E69" t="s">
-        <v>233</v>
+        <v>259</v>
       </c>
       <c r="F69" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>240</v>
-      </c>
-      <c r="B70" t="s">
-        <v>241</v>
+        <v>252</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>268</v>
       </c>
       <c r="C70" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="D70" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="E70" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="F70" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>193</v>
+        <v>253</v>
       </c>
       <c r="B71" t="s">
-        <v>194</v>
+        <v>274</v>
       </c>
       <c r="C71" t="s">
-        <v>195</v>
+        <v>248</v>
       </c>
       <c r="D71" t="s">
-        <v>195</v>
+        <v>248</v>
       </c>
       <c r="E71" t="s">
-        <v>196</v>
+        <v>261</v>
       </c>
       <c r="F71" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>222</v>
+        <v>254</v>
       </c>
       <c r="B72" t="s">
-        <v>223</v>
+        <v>273</v>
       </c>
       <c r="C72" t="s">
-        <v>195</v>
+        <v>248</v>
       </c>
       <c r="D72" t="s">
-        <v>195</v>
-      </c>
-      <c r="E72" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="F72" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>225</v>
-      </c>
-      <c r="B73" t="s">
-        <v>223</v>
+        <v>255</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>269</v>
       </c>
       <c r="C73" t="s">
-        <v>195</v>
+        <v>248</v>
       </c>
       <c r="D73" t="s">
-        <v>195</v>
-      </c>
-      <c r="E73" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="F73" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>5</v>
-      </c>
-      <c r="B74" t="s">
-        <v>6</v>
+        <v>256</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>266</v>
       </c>
       <c r="C74" t="s">
-        <v>7</v>
+        <v>248</v>
       </c>
       <c r="D74" t="s">
-        <v>8</v>
+        <v>248</v>
       </c>
       <c r="E74" t="s">
-        <v>9</v>
+        <v>262</v>
       </c>
       <c r="F74" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>10</v>
-      </c>
-      <c r="B75" t="s">
-        <v>11</v>
+        <v>263</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>270</v>
       </c>
       <c r="C75" t="s">
-        <v>7</v>
+        <v>248</v>
       </c>
       <c r="D75" t="s">
-        <v>8</v>
+        <v>248</v>
       </c>
       <c r="E75" t="s">
-        <v>12</v>
+        <v>267</v>
       </c>
       <c r="F75" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>83</v>
-      </c>
-      <c r="B76" t="s">
-        <v>84</v>
+        <v>264</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>270</v>
       </c>
       <c r="C76" t="s">
-        <v>85</v>
+        <v>248</v>
       </c>
       <c r="D76" t="s">
-        <v>8</v>
-      </c>
-      <c r="E76" t="s">
-        <v>86</v>
+        <v>248</v>
       </c>
       <c r="F76" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>95</v>
+        <v>41</v>
       </c>
       <c r="B77" t="s">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="C77" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="D77" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E77" t="s">
-        <v>97</v>
+        <v>44</v>
       </c>
       <c r="F77" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>153</v>
+        <v>110</v>
       </c>
       <c r="B78" t="s">
-        <v>154</v>
+        <v>111</v>
       </c>
       <c r="C78" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="D78" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E78" t="s">
-        <v>155</v>
+        <v>112</v>
       </c>
       <c r="F78" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>204</v>
+        <v>177</v>
       </c>
       <c r="B79" t="s">
-        <v>205</v>
+        <v>178</v>
       </c>
       <c r="C79" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="D79" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E79" t="s">
-        <v>206</v>
+        <v>282</v>
       </c>
       <c r="F79" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>207</v>
+        <v>226</v>
       </c>
       <c r="B80" t="s">
-        <v>208</v>
+        <v>227</v>
       </c>
       <c r="C80" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="D80" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E80" t="s">
-        <v>209</v>
+        <v>283</v>
       </c>
       <c r="F80" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>210</v>
+        <v>234</v>
       </c>
       <c r="B81" t="s">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="C81" t="s">
-        <v>7</v>
+        <v>43</v>
       </c>
       <c r="D81" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="E81" t="s">
-        <v>212</v>
+        <v>284</v>
       </c>
       <c r="F81" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>250</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>251</v>
+        <v>188</v>
+      </c>
+      <c r="B82" t="s">
+        <v>189</v>
       </c>
       <c r="C82" t="s">
-        <v>245</v>
+        <v>190</v>
       </c>
       <c r="D82" t="s">
-        <v>16</v>
+        <v>190</v>
       </c>
       <c r="E82" t="s">
-        <v>252</v>
+        <v>191</v>
       </c>
       <c r="F82" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>257</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>281</v>
+        <v>217</v>
+      </c>
+      <c r="B83" t="s">
+        <v>218</v>
       </c>
       <c r="C83" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="D83" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="E83" t="s">
-        <v>265</v>
+        <v>219</v>
       </c>
       <c r="F83" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>258</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>275</v>
+        <v>220</v>
+      </c>
+      <c r="B84" t="s">
+        <v>218</v>
       </c>
       <c r="C84" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="D84" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="E84" t="s">
-        <v>266</v>
+        <v>219</v>
       </c>
       <c r="F84" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>259</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>282</v>
+        <v>5</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="C85" t="s">
-        <v>256</v>
+        <v>7</v>
       </c>
       <c r="D85" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E85" t="s">
-        <v>267</v>
+        <v>9</v>
       </c>
       <c r="F85" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>260</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>278</v>
+        <v>10</v>
+      </c>
+      <c r="B86" t="s">
+        <v>11</v>
       </c>
       <c r="C86" t="s">
-        <v>256</v>
+        <v>7</v>
       </c>
       <c r="D86" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E86" t="s">
-        <v>268</v>
+        <v>12</v>
       </c>
       <c r="F86" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>261</v>
+        <v>82</v>
       </c>
       <c r="B87" t="s">
-        <v>284</v>
+        <v>83</v>
       </c>
       <c r="C87" t="s">
-        <v>256</v>
+        <v>84</v>
       </c>
       <c r="D87" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>269</v>
+        <v>85</v>
       </c>
       <c r="F87" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>262</v>
+        <v>94</v>
       </c>
       <c r="B88" t="s">
-        <v>283</v>
+        <v>95</v>
       </c>
       <c r="C88" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="D88" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E88" t="s">
-        <v>270</v>
+        <v>96</v>
       </c>
       <c r="F88" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>263</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>279</v>
+        <v>151</v>
+      </c>
+      <c r="B89" t="s">
+        <v>152</v>
       </c>
       <c r="C89" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="D89" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E89" t="s">
-        <v>271</v>
+        <v>153</v>
       </c>
       <c r="F89" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>264</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>276</v>
+        <v>199</v>
+      </c>
+      <c r="B90" t="s">
+        <v>200</v>
       </c>
       <c r="C90" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="D90" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E90" t="s">
-        <v>272</v>
+        <v>201</v>
       </c>
       <c r="F90" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>273</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>280</v>
+        <v>202</v>
+      </c>
+      <c r="B91" t="s">
+        <v>203</v>
       </c>
       <c r="C91" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="D91" t="s">
-        <v>256</v>
+        <v>8</v>
       </c>
       <c r="E91" t="s">
-        <v>277</v>
+        <v>204</v>
       </c>
       <c r="F91" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>274</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>280</v>
+        <v>205</v>
+      </c>
+      <c r="B92" t="s">
+        <v>206</v>
       </c>
       <c r="C92" t="s">
-        <v>256</v>
+        <v>7</v>
       </c>
       <c r="D92" t="s">
-        <v>256</v>
+        <v>8</v>
+      </c>
+      <c r="E92" t="s">
+        <v>207</v>
       </c>
       <c r="F92" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B31" r:id="rId1" xr:uid="{980DC69E-AE68-4641-91F2-05169A270488}"/>
-    <hyperlink ref="B52" r:id="rId2" xr:uid="{E6943F17-6C80-4605-A40B-053F9F734E11}"/>
-    <hyperlink ref="B54" r:id="rId3" xr:uid="{7DF46576-4CF8-4C0A-8982-315AE05E9433}"/>
-    <hyperlink ref="B82" r:id="rId4" xr:uid="{526DC027-CD0E-4347-8477-5DD3919072C9}"/>
-    <hyperlink ref="B84" r:id="rId5" xr:uid="{05BE8DF4-EE01-44FC-9F5F-A59CBF58993C}"/>
-    <hyperlink ref="B90" r:id="rId6" xr:uid="{2BD72C8A-46C6-4AA2-97FF-3C59E480CFF9}"/>
-    <hyperlink ref="B89" r:id="rId7" xr:uid="{6DEF3BD0-5D4D-487E-9A78-0E628D8E12C8}"/>
-    <hyperlink ref="B91" r:id="rId8" xr:uid="{2ECEB650-EA1C-4977-A07D-E1F44E63FDA5}"/>
-    <hyperlink ref="B83" r:id="rId9" xr:uid="{4BB4CE27-95D2-4BD8-A8AE-22D0AB4F1D12}"/>
-    <hyperlink ref="B92" r:id="rId10" xr:uid="{CCB7569F-7C4A-45AC-A738-5A7777A8BD12}"/>
-    <hyperlink ref="B86" r:id="rId11" xr:uid="{6F9ECF71-34EB-4E87-B39B-A5F3CB72547F}"/>
-    <hyperlink ref="B85" r:id="rId12" xr:uid="{AE447FCE-5475-4563-A677-E467C73C7B97}"/>
+    <hyperlink ref="B53" r:id="rId2" xr:uid="{E6943F17-6C80-4605-A40B-053F9F734E11}"/>
+    <hyperlink ref="B55" r:id="rId3" xr:uid="{7DF46576-4CF8-4C0A-8982-315AE05E9433}"/>
+    <hyperlink ref="B39" r:id="rId4" xr:uid="{526DC027-CD0E-4347-8477-5DD3919072C9}"/>
+    <hyperlink ref="B68" r:id="rId5" xr:uid="{05BE8DF4-EE01-44FC-9F5F-A59CBF58993C}"/>
+    <hyperlink ref="B74" r:id="rId6" xr:uid="{2BD72C8A-46C6-4AA2-97FF-3C59E480CFF9}"/>
+    <hyperlink ref="B73" r:id="rId7" xr:uid="{6DEF3BD0-5D4D-487E-9A78-0E628D8E12C8}"/>
+    <hyperlink ref="B75" r:id="rId8" xr:uid="{2ECEB650-EA1C-4977-A07D-E1F44E63FDA5}"/>
+    <hyperlink ref="B67" r:id="rId9" xr:uid="{4BB4CE27-95D2-4BD8-A8AE-22D0AB4F1D12}"/>
+    <hyperlink ref="B76" r:id="rId10" xr:uid="{CCB7569F-7C4A-45AC-A738-5A7777A8BD12}"/>
+    <hyperlink ref="B70" r:id="rId11" xr:uid="{6F9ECF71-34EB-4E87-B39B-A5F3CB72547F}"/>
+    <hyperlink ref="B69" r:id="rId12" xr:uid="{AE447FCE-5475-4563-A677-E467C73C7B97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>

<commit_message>
se exporta el doc de resguardo
</commit_message>
<xml_diff>
--- a/src/assets/Usuarios de crownparadise.xlsx
+++ b/src/assets/Usuarios de crownparadise.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E460E8-0B8E-4F1D-8A4B-009CEED57766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930FAAD9-3D1B-4D66-A2BA-05E756D74041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="288">
   <si>
     <t>Nombre</t>
   </si>
@@ -137,9 +137,6 @@
     <t>rechumanos1@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\capacitacion</t>
-  </si>
-  <si>
     <t>Asunción Ventura Jimenez</t>
   </si>
   <si>
@@ -149,9 +146,6 @@
     <t>Mantenimiento</t>
   </si>
   <si>
-    <t>CROWNCUN\jefemanto</t>
-  </si>
-  <si>
     <t>Auxiliar Administrativo</t>
   </si>
   <si>
@@ -314,9 +308,6 @@
     <t>crownclub@crownparadise.com</t>
   </si>
   <si>
-    <t>ARRIVA\crowncluncun</t>
-  </si>
-  <si>
     <t>Disco Nitro</t>
   </si>
   <si>
@@ -524,9 +515,6 @@
     <t>cpc-nominas@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\nominas</t>
-  </si>
-  <si>
     <t>Marcos Dolores</t>
   </si>
   <si>
@@ -707,18 +695,12 @@
     <t>luzysonido@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\luzysonido</t>
-  </si>
-  <si>
     <t>Toma Ordenes Ama de Llaves</t>
   </si>
   <si>
     <t>amallaves-cun@crownparadise.com</t>
   </si>
   <si>
-    <t>CROWNCUN\amadellaves2</t>
-  </si>
-  <si>
     <t>Toma Ordenes Mantenimiento</t>
   </si>
   <si>
@@ -870,6 +852,33 @@
   </si>
   <si>
     <t>ARRIVA\mantenimientocun02</t>
+  </si>
+  <si>
+    <t>ARRIVA\aydcun01</t>
+  </si>
+  <si>
+    <t>Teatro Laptop</t>
+  </si>
+  <si>
+    <t>ARRIVA\aydcun02</t>
+  </si>
+  <si>
+    <t>ARRIVA\capacun01</t>
+  </si>
+  <si>
+    <t>ARRIVA\nominascun</t>
+  </si>
+  <si>
+    <t>ARRIVA\crownclubcun</t>
+  </si>
+  <si>
+    <t>ARRIVA\amallavescun01</t>
+  </si>
+  <si>
+    <t>ARRIVA\jefemantocun</t>
+  </si>
+  <si>
+    <t>ARRIVA\spacun01</t>
   </si>
 </sst>
 </file>
@@ -907,27 +916,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -945,7 +939,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -983,10 +977,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}" name="Tabla1" displayName="Tabla1" ref="A1:F92" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:F92" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F92">
-    <sortCondition ref="D1:D92"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}" name="Tabla1" displayName="Tabla1" ref="A1:F93" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:F93" xr:uid="{A9299B97-B99B-4DC8-8282-36BE7801C421}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F93">
+    <sortCondition ref="D1:D93"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{9490AABE-096E-46D2-A730-536117DCF14A}" name="Nombre"/>
@@ -1323,7 +1317,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -1350,127 +1344,127 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E2" t="s">
         <v>113</v>
       </c>
-      <c r="B2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E2" t="s">
-        <v>116</v>
-      </c>
       <c r="F2" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F3" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F4" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E5" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="F5" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B6" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E6" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="F6" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B7" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D7" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E7" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="F7" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1490,15 +1484,15 @@
         <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -1507,15 +1501,15 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B10" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
@@ -1524,18 +1518,15 @@
         <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="F10" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>228</v>
-      </c>
-      <c r="B11" t="s">
-        <v>229</v>
+        <v>280</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -1544,38 +1535,38 @@
         <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>230</v>
+        <v>281</v>
       </c>
       <c r="F11" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>224</v>
       </c>
       <c r="B12" t="s">
-        <v>28</v>
+        <v>225</v>
       </c>
       <c r="C12" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F12" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>29</v>
@@ -1584,18 +1575,18 @@
         <v>29</v>
       </c>
       <c r="E13" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="F13" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
         <v>29</v>
@@ -1604,18 +1595,18 @@
         <v>29</v>
       </c>
       <c r="E14" t="s">
-        <v>77</v>
+        <v>275</v>
       </c>
       <c r="F14" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>141</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="C15" t="s">
         <v>29</v>
@@ -1624,18 +1615,18 @@
         <v>29</v>
       </c>
       <c r="E15" t="s">
-        <v>143</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>139</v>
       </c>
       <c r="C16" t="s">
         <v>29</v>
@@ -1644,18 +1635,18 @@
         <v>29</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>140</v>
       </c>
       <c r="F16" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B17" t="s">
-        <v>156</v>
+        <v>98</v>
       </c>
       <c r="C17" t="s">
         <v>29</v>
@@ -1664,38 +1655,38 @@
         <v>29</v>
       </c>
       <c r="E17" t="s">
-        <v>157</v>
+        <v>282</v>
       </c>
       <c r="F17" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>152</v>
       </c>
       <c r="B18" t="s">
-        <v>14</v>
+        <v>153</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E18" t="s">
-        <v>17</v>
+        <v>154</v>
       </c>
       <c r="F18" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C19" t="s">
         <v>15</v>
@@ -1704,58 +1695,58 @@
         <v>16</v>
       </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="F20" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B21" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D21" t="s">
         <v>16</v>
       </c>
       <c r="E21" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="F21" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C22" t="s">
         <v>15</v>
@@ -1764,18 +1755,18 @@
         <v>16</v>
       </c>
       <c r="E22" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F22" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="C23" t="s">
         <v>15</v>
@@ -1784,78 +1775,78 @@
         <v>16</v>
       </c>
       <c r="E23" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="F23" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="D24" t="s">
         <v>16</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="F24" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D25" t="s">
         <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="D26" t="s">
         <v>16</v>
       </c>
       <c r="E26" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="F26" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="B27" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C27" t="s">
         <v>15</v>
@@ -1864,118 +1855,118 @@
         <v>16</v>
       </c>
       <c r="E27" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="F27" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B28" t="s">
-        <v>124</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>125</v>
+        <v>15</v>
       </c>
       <c r="D28" t="s">
         <v>16</v>
       </c>
       <c r="E28" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="F28" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="B29" t="s">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="C29" t="s">
-        <v>32</v>
+        <v>122</v>
       </c>
       <c r="D29" t="s">
         <v>16</v>
       </c>
       <c r="E29" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B30" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C30" t="s">
-        <v>146</v>
+        <v>32</v>
       </c>
       <c r="D30" t="s">
         <v>16</v>
       </c>
       <c r="E30" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="F30" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>240</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>241</v>
+        <v>141</v>
+      </c>
+      <c r="B31" t="s">
+        <v>142</v>
       </c>
       <c r="C31" t="s">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="D31" t="s">
         <v>16</v>
       </c>
       <c r="E31" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="F31" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>164</v>
-      </c>
-      <c r="B32" t="s">
-        <v>165</v>
+        <v>234</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>235</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="D32" t="s">
         <v>16</v>
       </c>
       <c r="E32" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F32" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B33" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C33" t="s">
         <v>15</v>
@@ -1984,155 +1975,155 @@
         <v>16</v>
       </c>
       <c r="E33" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F33" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B34" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C34" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="D34" t="s">
         <v>16</v>
       </c>
       <c r="E34" t="s">
-        <v>176</v>
+        <v>283</v>
       </c>
       <c r="F34" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="B35" t="s">
-        <v>101</v>
+        <v>171</v>
       </c>
       <c r="C35" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="D35" t="s">
         <v>16</v>
       </c>
       <c r="E35" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="F35" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>208</v>
+        <v>175</v>
       </c>
       <c r="B36" t="s">
-        <v>209</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>146</v>
+        <v>15</v>
       </c>
       <c r="D36" t="s">
         <v>16</v>
       </c>
       <c r="E36" t="s">
-        <v>210</v>
+        <v>176</v>
       </c>
       <c r="F36" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B37" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C37" t="s">
-        <v>15</v>
+        <v>143</v>
       </c>
       <c r="D37" t="s">
         <v>16</v>
       </c>
       <c r="E37" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="F37" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>236</v>
+        <v>210</v>
       </c>
       <c r="B38" t="s">
-        <v>237</v>
+        <v>211</v>
       </c>
       <c r="C38" t="s">
-        <v>238</v>
+        <v>15</v>
       </c>
       <c r="D38" t="s">
         <v>16</v>
       </c>
       <c r="E38" t="s">
-        <v>239</v>
+        <v>212</v>
       </c>
       <c r="F38" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>243</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>244</v>
+        <v>230</v>
+      </c>
+      <c r="B39" t="s">
+        <v>231</v>
       </c>
       <c r="C39" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="D39" t="s">
         <v>16</v>
       </c>
+      <c r="E39" t="s">
+        <v>233</v>
+      </c>
       <c r="F39" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>21</v>
-      </c>
-      <c r="B40" t="s">
-        <v>22</v>
+        <v>237</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>238</v>
       </c>
       <c r="C40" t="s">
-        <v>23</v>
+        <v>232</v>
       </c>
       <c r="D40" t="s">
-        <v>24</v>
-      </c>
-      <c r="E40" t="s">
-        <v>277</v>
+        <v>16</v>
       </c>
       <c r="F40" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B41" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C41" t="s">
         <v>23</v>
@@ -2141,883 +2132,883 @@
         <v>24</v>
       </c>
       <c r="E41" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="F41" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="C42" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="D42" t="s">
         <v>24</v>
       </c>
       <c r="E42" t="s">
-        <v>54</v>
+        <v>270</v>
       </c>
       <c r="F42" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B43" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C43" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D43" t="s">
         <v>24</v>
       </c>
       <c r="E43" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F43" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D44" t="s">
         <v>24</v>
       </c>
       <c r="E44" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F44" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B45" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C45" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D45" t="s">
         <v>24</v>
       </c>
       <c r="E45" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F45" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B46" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C46" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D46" t="s">
         <v>24</v>
       </c>
       <c r="E46" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F46" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B47" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C47" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D47" t="s">
         <v>24</v>
       </c>
       <c r="E47" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F47" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B48" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C48" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="D48" t="s">
         <v>24</v>
       </c>
       <c r="E48" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F48" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="B49" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="C49" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D49" t="s">
         <v>24</v>
       </c>
       <c r="E49" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="F49" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="B50" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D50" t="s">
         <v>24</v>
       </c>
       <c r="E50" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="F50" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C51" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D51" t="s">
         <v>24</v>
       </c>
       <c r="E51" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F51" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B52" t="s">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="C52" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D52" t="s">
         <v>24</v>
       </c>
       <c r="E52" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="F52" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>108</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>242</v>
+        <v>95</v>
+      </c>
+      <c r="B53" t="s">
+        <v>96</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>65</v>
       </c>
       <c r="D53" t="s">
         <v>24</v>
       </c>
       <c r="E53" t="s">
-        <v>109</v>
+        <v>284</v>
       </c>
       <c r="F53" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>117</v>
-      </c>
-      <c r="B54" t="s">
-        <v>118</v>
+        <v>105</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>236</v>
       </c>
       <c r="C54" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="D54" t="s">
         <v>24</v>
       </c>
       <c r="E54" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F54" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>130</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>73</v>
+        <v>114</v>
+      </c>
+      <c r="B55" t="s">
+        <v>115</v>
       </c>
       <c r="C55" t="s">
-        <v>53</v>
+        <v>24</v>
       </c>
       <c r="D55" t="s">
         <v>24</v>
       </c>
       <c r="E55" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="F55" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>134</v>
-      </c>
-      <c r="B56" t="s">
-        <v>135</v>
+        <v>127</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>71</v>
       </c>
       <c r="C56" t="s">
-        <v>136</v>
+        <v>51</v>
       </c>
       <c r="D56" t="s">
         <v>24</v>
       </c>
       <c r="E56" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="F56" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>148</v>
+        <v>131</v>
       </c>
       <c r="B57" t="s">
-        <v>101</v>
+        <v>132</v>
       </c>
       <c r="C57" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D57" t="s">
         <v>24</v>
       </c>
       <c r="E57" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="F57" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="B58" t="s">
-        <v>159</v>
+        <v>98</v>
       </c>
       <c r="C58" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D58" t="s">
         <v>24</v>
       </c>
       <c r="E58" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="F58" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B59" t="s">
-        <v>101</v>
+        <v>156</v>
       </c>
       <c r="C59" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D59" t="s">
         <v>24</v>
       </c>
+      <c r="E59" t="s">
+        <v>157</v>
+      </c>
       <c r="F59" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B60" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D60" t="s">
         <v>24</v>
       </c>
       <c r="F60" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="B61" t="s">
-        <v>171</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
-        <v>172</v>
+        <v>146</v>
       </c>
       <c r="D61" t="s">
         <v>24</v>
       </c>
-      <c r="E61" t="s">
-        <v>173</v>
-      </c>
       <c r="F61" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>185</v>
+        <v>166</v>
       </c>
       <c r="B62" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="C62" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="D62" t="s">
         <v>24</v>
       </c>
-      <c r="E62" s="3" t="s">
-        <v>279</v>
+      <c r="E62" t="s">
+        <v>169</v>
       </c>
       <c r="F62" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>223</v>
+        <v>181</v>
       </c>
       <c r="B63" t="s">
-        <v>224</v>
+        <v>182</v>
       </c>
       <c r="C63" t="s">
-        <v>53</v>
+        <v>183</v>
       </c>
       <c r="D63" t="s">
         <v>24</v>
       </c>
-      <c r="E63" t="s">
-        <v>225</v>
+      <c r="E63" s="3" t="s">
+        <v>273</v>
       </c>
       <c r="F63" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="B64" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="C64" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="D64" t="s">
         <v>24</v>
       </c>
       <c r="E64" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="F64" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>181</v>
+        <v>226</v>
       </c>
       <c r="B65" t="s">
-        <v>182</v>
+        <v>227</v>
       </c>
       <c r="C65" t="s">
-        <v>183</v>
+        <v>23</v>
       </c>
       <c r="D65" t="s">
-        <v>183</v>
+        <v>24</v>
       </c>
       <c r="E65" t="s">
-        <v>184</v>
+        <v>285</v>
       </c>
       <c r="F65" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>195</v>
+        <v>177</v>
       </c>
       <c r="B66" t="s">
-        <v>196</v>
+        <v>178</v>
       </c>
       <c r="C66" t="s">
-        <v>197</v>
+        <v>179</v>
       </c>
       <c r="D66" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E66" t="s">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="F66" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>249</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>271</v>
+        <v>191</v>
+      </c>
+      <c r="B67" t="s">
+        <v>192</v>
       </c>
       <c r="C67" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="D67" t="s">
-        <v>248</v>
+        <v>179</v>
       </c>
       <c r="E67" t="s">
-        <v>257</v>
+        <v>194</v>
       </c>
       <c r="F67" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="B68" s="2" t="s">
         <v>265</v>
       </c>
       <c r="C68" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D68" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E68" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="F68" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>251</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>272</v>
+        <v>244</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>259</v>
       </c>
       <c r="C69" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D69" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E69" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="F69" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>252</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>268</v>
+        <v>245</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>266</v>
       </c>
       <c r="C70" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D70" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E70" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="F70" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>253</v>
-      </c>
-      <c r="B71" t="s">
-        <v>274</v>
+        <v>246</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>262</v>
       </c>
       <c r="C71" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D71" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E71" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="F71" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="B72" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="C72" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D72" t="s">
-        <v>248</v>
+        <v>242</v>
+      </c>
+      <c r="E72" t="s">
+        <v>255</v>
       </c>
       <c r="F72" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>255</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>269</v>
+        <v>248</v>
+      </c>
+      <c r="B73" t="s">
+        <v>267</v>
       </c>
       <c r="C73" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D73" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="F73" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C74" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D74" t="s">
-        <v>248</v>
-      </c>
-      <c r="E74" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="F74" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>263</v>
+        <v>250</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="C75" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D75" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E75" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="F75" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>257</v>
+      </c>
+      <c r="B76" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="B76" s="2" t="s">
-        <v>270</v>
-      </c>
       <c r="C76" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="D76" t="s">
-        <v>248</v>
+        <v>242</v>
+      </c>
+      <c r="E76" t="s">
+        <v>261</v>
       </c>
       <c r="F76" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>41</v>
-      </c>
-      <c r="B77" t="s">
-        <v>42</v>
+        <v>258</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>264</v>
       </c>
       <c r="C77" t="s">
-        <v>43</v>
+        <v>242</v>
       </c>
       <c r="D77" t="s">
-        <v>43</v>
-      </c>
-      <c r="E77" t="s">
-        <v>44</v>
+        <v>242</v>
       </c>
       <c r="F77" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="B78" t="s">
-        <v>111</v>
+        <v>41</v>
       </c>
       <c r="C78" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D78" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E78" t="s">
-        <v>112</v>
+        <v>286</v>
       </c>
       <c r="F78" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>177</v>
+        <v>107</v>
       </c>
       <c r="B79" t="s">
-        <v>178</v>
+        <v>108</v>
       </c>
       <c r="C79" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D79" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E79" t="s">
-        <v>282</v>
+        <v>109</v>
       </c>
       <c r="F79" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>226</v>
+        <v>173</v>
       </c>
       <c r="B80" t="s">
-        <v>227</v>
+        <v>174</v>
       </c>
       <c r="C80" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D80" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E80" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="F80" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="B81" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="C81" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D81" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E81" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="F81" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>188</v>
+        <v>228</v>
       </c>
       <c r="B82" t="s">
-        <v>189</v>
+        <v>229</v>
       </c>
       <c r="C82" t="s">
-        <v>190</v>
+        <v>42</v>
       </c>
       <c r="D82" t="s">
-        <v>190</v>
+        <v>42</v>
       </c>
       <c r="E82" t="s">
-        <v>191</v>
+        <v>278</v>
       </c>
       <c r="F82" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="B83" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="C83" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D83" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E83" t="s">
-        <v>219</v>
+        <v>187</v>
       </c>
       <c r="F83" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B84" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C84" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D84" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E84" t="s">
-        <v>219</v>
+        <v>287</v>
       </c>
       <c r="F84" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>5</v>
-      </c>
-      <c r="B85" s="5" t="s">
-        <v>6</v>
+        <v>216</v>
+      </c>
+      <c r="B85" t="s">
+        <v>214</v>
       </c>
       <c r="C85" t="s">
-        <v>7</v>
+        <v>186</v>
       </c>
       <c r="D85" t="s">
-        <v>8</v>
+        <v>186</v>
       </c>
       <c r="E85" t="s">
-        <v>9</v>
+        <v>215</v>
       </c>
       <c r="F85" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>10</v>
-      </c>
-      <c r="B86" t="s">
-        <v>11</v>
+        <v>5</v>
+      </c>
+      <c r="B86" s="5" t="s">
+        <v>6</v>
       </c>
       <c r="C86" t="s">
         <v>7</v>
@@ -3026,58 +3017,58 @@
         <v>8</v>
       </c>
       <c r="E86" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F86" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="B87" t="s">
-        <v>83</v>
+        <v>11</v>
       </c>
       <c r="C87" t="s">
-        <v>84</v>
+        <v>7</v>
       </c>
       <c r="D87" t="s">
         <v>8</v>
       </c>
       <c r="E87" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="F87" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="B88" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="C88" t="s">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="D88" t="s">
         <v>8</v>
       </c>
       <c r="E88" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="F88" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>151</v>
+        <v>92</v>
       </c>
       <c r="B89" t="s">
-        <v>152</v>
+        <v>93</v>
       </c>
       <c r="C89" t="s">
         <v>8</v>
@@ -3086,18 +3077,18 @@
         <v>8</v>
       </c>
       <c r="E89" t="s">
-        <v>153</v>
+        <v>94</v>
       </c>
       <c r="F89" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>199</v>
+        <v>148</v>
       </c>
       <c r="B90" t="s">
-        <v>200</v>
+        <v>149</v>
       </c>
       <c r="C90" t="s">
         <v>8</v>
@@ -3106,18 +3097,18 @@
         <v>8</v>
       </c>
       <c r="E90" t="s">
-        <v>201</v>
+        <v>150</v>
       </c>
       <c r="F90" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B91" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C91" t="s">
         <v>8</v>
@@ -3126,46 +3117,66 @@
         <v>8</v>
       </c>
       <c r="E91" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="F91" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B92" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="C92" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D92" t="s">
         <v>8</v>
       </c>
       <c r="E92" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="F92" t="s">
-        <v>246</v>
+        <v>240</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>201</v>
+      </c>
+      <c r="B93" t="s">
+        <v>202</v>
+      </c>
+      <c r="C93" t="s">
+        <v>7</v>
+      </c>
+      <c r="D93" t="s">
+        <v>8</v>
+      </c>
+      <c r="E93" t="s">
+        <v>203</v>
+      </c>
+      <c r="F93" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B31" r:id="rId1" xr:uid="{980DC69E-AE68-4641-91F2-05169A270488}"/>
-    <hyperlink ref="B53" r:id="rId2" xr:uid="{E6943F17-6C80-4605-A40B-053F9F734E11}"/>
-    <hyperlink ref="B55" r:id="rId3" xr:uid="{7DF46576-4CF8-4C0A-8982-315AE05E9433}"/>
-    <hyperlink ref="B39" r:id="rId4" xr:uid="{526DC027-CD0E-4347-8477-5DD3919072C9}"/>
-    <hyperlink ref="B68" r:id="rId5" xr:uid="{05BE8DF4-EE01-44FC-9F5F-A59CBF58993C}"/>
-    <hyperlink ref="B74" r:id="rId6" xr:uid="{2BD72C8A-46C6-4AA2-97FF-3C59E480CFF9}"/>
-    <hyperlink ref="B73" r:id="rId7" xr:uid="{6DEF3BD0-5D4D-487E-9A78-0E628D8E12C8}"/>
-    <hyperlink ref="B75" r:id="rId8" xr:uid="{2ECEB650-EA1C-4977-A07D-E1F44E63FDA5}"/>
-    <hyperlink ref="B67" r:id="rId9" xr:uid="{4BB4CE27-95D2-4BD8-A8AE-22D0AB4F1D12}"/>
-    <hyperlink ref="B76" r:id="rId10" xr:uid="{CCB7569F-7C4A-45AC-A738-5A7777A8BD12}"/>
-    <hyperlink ref="B70" r:id="rId11" xr:uid="{6F9ECF71-34EB-4E87-B39B-A5F3CB72547F}"/>
-    <hyperlink ref="B69" r:id="rId12" xr:uid="{AE447FCE-5475-4563-A677-E467C73C7B97}"/>
+    <hyperlink ref="B32" r:id="rId1" xr:uid="{980DC69E-AE68-4641-91F2-05169A270488}"/>
+    <hyperlink ref="B54" r:id="rId2" xr:uid="{E6943F17-6C80-4605-A40B-053F9F734E11}"/>
+    <hyperlink ref="B56" r:id="rId3" xr:uid="{7DF46576-4CF8-4C0A-8982-315AE05E9433}"/>
+    <hyperlink ref="B40" r:id="rId4" xr:uid="{526DC027-CD0E-4347-8477-5DD3919072C9}"/>
+    <hyperlink ref="B69" r:id="rId5" xr:uid="{05BE8DF4-EE01-44FC-9F5F-A59CBF58993C}"/>
+    <hyperlink ref="B75" r:id="rId6" xr:uid="{2BD72C8A-46C6-4AA2-97FF-3C59E480CFF9}"/>
+    <hyperlink ref="B74" r:id="rId7" xr:uid="{6DEF3BD0-5D4D-487E-9A78-0E628D8E12C8}"/>
+    <hyperlink ref="B76" r:id="rId8" xr:uid="{2ECEB650-EA1C-4977-A07D-E1F44E63FDA5}"/>
+    <hyperlink ref="B68" r:id="rId9" xr:uid="{4BB4CE27-95D2-4BD8-A8AE-22D0AB4F1D12}"/>
+    <hyperlink ref="B77" r:id="rId10" xr:uid="{CCB7569F-7C4A-45AC-A738-5A7777A8BD12}"/>
+    <hyperlink ref="B71" r:id="rId11" xr:uid="{6F9ECF71-34EB-4E87-B39B-A5F3CB72547F}"/>
+    <hyperlink ref="B70" r:id="rId12" xr:uid="{AE447FCE-5475-4563-A677-E467C73C7B97}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>

</xml_diff>